<commit_message>
feature/fsel-5423: Update Export File
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoKetQuaHocTapAca.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoKetQuaHocTapAca.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PhanPhuc\Fsel\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ManagerReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{156935BA-9A8E-4118-B64B-7F90246922BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC015000-7834-4D5B-9BB2-DA423E8F885D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C9B9EFB7-A784-4396-91D6-1A13258A8575}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C9B9EFB7-A784-4396-91D6-1A13258A8575}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="63">
   <si>
     <t>BÁO CÁO KẾT QUẢ HỌC TẬP (Academic)</t>
   </si>
@@ -211,6 +211,9 @@
   </si>
   <si>
     <t>Unit 12 : {0}</t>
+  </si>
+  <si>
+    <t>UserName</t>
   </si>
 </sst>
 </file>
@@ -399,28 +402,28 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -735,287 +738,291 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F296DC0F-8D5A-4FA7-96B9-2C09CA3840C7}">
-  <dimension ref="A1:Y9"/>
+  <dimension ref="A1:Z9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15" style="19" customWidth="1"/>
-    <col min="2" max="2" width="14.75" style="19" customWidth="1"/>
-    <col min="3" max="3" width="15.625" style="19" customWidth="1"/>
-    <col min="4" max="4" width="9" style="19"/>
-    <col min="5" max="5" width="17.125" style="19" customWidth="1"/>
-    <col min="6" max="6" width="25.375" style="19" customWidth="1"/>
-    <col min="7" max="7" width="22.25" style="19" customWidth="1"/>
-    <col min="8" max="8" width="21.125" style="19" customWidth="1"/>
-    <col min="9" max="9" width="20.75" style="19" customWidth="1"/>
-    <col min="10" max="10" width="22" style="19" customWidth="1"/>
-    <col min="11" max="11" width="29" style="19" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.125" style="19" customWidth="1"/>
-    <col min="13" max="13" width="25.125" style="19" customWidth="1"/>
-    <col min="14" max="14" width="20.375" style="19" customWidth="1"/>
-    <col min="15" max="16" width="23.125" style="19" customWidth="1"/>
-    <col min="17" max="17" width="22" style="19" customWidth="1"/>
-    <col min="18" max="18" width="21.75" style="19" customWidth="1"/>
-    <col min="19" max="19" width="20.875" style="19" customWidth="1"/>
-    <col min="20" max="20" width="19.375" style="19" customWidth="1"/>
-    <col min="21" max="21" width="20.875" style="19" customWidth="1"/>
-    <col min="22" max="22" width="13" style="19" customWidth="1"/>
-    <col min="23" max="23" width="20" style="19" customWidth="1"/>
-    <col min="24" max="16384" width="9" style="19"/>
+    <col min="1" max="2" width="15" style="12" customWidth="1"/>
+    <col min="3" max="3" width="14.75" style="12" customWidth="1"/>
+    <col min="4" max="4" width="15.625" style="12" customWidth="1"/>
+    <col min="5" max="5" width="9" style="12"/>
+    <col min="6" max="6" width="17.125" style="12" customWidth="1"/>
+    <col min="7" max="7" width="25.375" style="12" customWidth="1"/>
+    <col min="8" max="8" width="22.25" style="12" customWidth="1"/>
+    <col min="9" max="9" width="21.125" style="12" customWidth="1"/>
+    <col min="10" max="10" width="20.75" style="12" customWidth="1"/>
+    <col min="11" max="11" width="22" style="12" customWidth="1"/>
+    <col min="12" max="12" width="29" style="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="29.125" style="12" customWidth="1"/>
+    <col min="14" max="14" width="25.125" style="12" customWidth="1"/>
+    <col min="15" max="15" width="20.375" style="12" customWidth="1"/>
+    <col min="16" max="17" width="23.125" style="12" customWidth="1"/>
+    <col min="18" max="18" width="22" style="12" customWidth="1"/>
+    <col min="19" max="19" width="21.75" style="12" customWidth="1"/>
+    <col min="20" max="20" width="20.875" style="12" customWidth="1"/>
+    <col min="21" max="21" width="19.375" style="12" customWidth="1"/>
+    <col min="22" max="22" width="20.875" style="12" customWidth="1"/>
+    <col min="23" max="23" width="13" style="12" customWidth="1"/>
+    <col min="24" max="24" width="20" style="12" customWidth="1"/>
+    <col min="25" max="16384" width="9" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:26" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="T1" s="16"/>
-      <c r="U1" s="16"/>
-      <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
-      <c r="X1" s="16"/>
-      <c r="Y1" s="16"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="W1" s="14"/>
+      <c r="X1" s="14"/>
+      <c r="Y1" s="14"/>
+      <c r="Z1" s="14"/>
     </row>
-    <row r="2" spans="1:25" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="6" t="s">
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="K2" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="L2" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="M2" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="N2" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="N2" s="6"/>
       <c r="O2" s="6"/>
-      <c r="P2" s="7"/>
+      <c r="P2" s="6"/>
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
-      <c r="S2" s="1"/>
+      <c r="S2" s="7"/>
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
-      <c r="Y2" s="2"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="2"/>
     </row>
-    <row r="3" spans="1:25" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="6">
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="6">
         <v>120</v>
       </c>
-      <c r="G3" s="6"/>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="7"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="10"/>
       <c r="P3" s="7"/>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
-      <c r="S3" s="1"/>
+      <c r="S3" s="7"/>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
       <c r="W3" s="1"/>
       <c r="X3" s="1"/>
-      <c r="Y3" s="2"/>
+      <c r="Y3" s="1"/>
+      <c r="Z3" s="2"/>
     </row>
-    <row r="4" spans="1:25" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+    <row r="4" spans="1:26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="6" t="s">
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="E4" s="16"/>
+      <c r="F4" s="16"/>
+      <c r="G4" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="K4" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="L4" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L4" s="6"/>
       <c r="M4" s="6"/>
-      <c r="N4" s="10"/>
-      <c r="O4" s="7"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="10"/>
       <c r="P4" s="7"/>
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
-      <c r="S4" s="1"/>
+      <c r="S4" s="7"/>
       <c r="T4" s="1"/>
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="2"/>
+      <c r="Y4" s="1"/>
+      <c r="Z4" s="2"/>
     </row>
-    <row r="5" spans="1:25" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+    <row r="5" spans="1:26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="6" t="s">
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="6"/>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
       <c r="M5" s="6"/>
-      <c r="N5" s="10"/>
-      <c r="O5" s="7"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="10"/>
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
-      <c r="S5" s="1"/>
+      <c r="S5" s="7"/>
       <c r="T5" s="1"/>
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
       <c r="W5" s="1"/>
       <c r="X5" s="1"/>
-      <c r="Y5" s="2"/>
+      <c r="Y5" s="1"/>
+      <c r="Z5" s="2"/>
     </row>
-    <row r="6" spans="1:25" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="18" t="s">
+    <row r="6" spans="1:26" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="8" t="s">
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="H6" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="I6" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="J6" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="K6" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="L6" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="L6" s="8" t="s">
+      <c r="M6" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="M6" s="8" t="s">
+      <c r="N6" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="N6" s="6" t="s">
+      <c r="O6" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="O6" s="8" t="s">
+      <c r="P6" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="P6" s="8" t="s">
+      <c r="Q6" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="Q6" s="8" t="s">
+      <c r="R6" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="R6" s="8"/>
-      <c r="S6" s="13"/>
-      <c r="T6" s="13"/>
-      <c r="U6" s="13"/>
-      <c r="V6" s="13"/>
-      <c r="W6" s="13"/>
-      <c r="X6" s="13"/>
-      <c r="Y6" s="14"/>
+      <c r="S6" s="8"/>
+      <c r="T6" s="18"/>
+      <c r="U6" s="18"/>
+      <c r="V6" s="18"/>
+      <c r="W6" s="18"/>
+      <c r="X6" s="18"/>
+      <c r="Y6" s="18"/>
+      <c r="Z6" s="19"/>
     </row>
-    <row r="7" spans="1:25" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="18"/>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="8" t="s">
+    <row r="7" spans="1:26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="17"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="I7" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="J7" s="8" t="s">
+      <c r="K7" s="8" t="s">
         <v>33</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>34</v>
       </c>
       <c r="L7" s="8" t="s">
         <v>34</v>
@@ -1023,10 +1030,10 @@
       <c r="M7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="N7" s="6" t="s">
+      <c r="N7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="O7" s="8" t="s">
+      <c r="O7" s="6" t="s">
         <v>34</v>
       </c>
       <c r="P7" s="8" t="s">
@@ -1035,133 +1042,140 @@
       <c r="Q7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="R7" s="8"/>
-      <c r="S7" s="13"/>
-      <c r="T7" s="13"/>
-      <c r="U7" s="13"/>
-      <c r="V7" s="13"/>
-      <c r="W7" s="13"/>
-      <c r="X7" s="13"/>
-      <c r="Y7" s="14"/>
+      <c r="R7" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="S7" s="8"/>
+      <c r="T7" s="18"/>
+      <c r="U7" s="18"/>
+      <c r="V7" s="18"/>
+      <c r="W7" s="18"/>
+      <c r="X7" s="18"/>
+      <c r="Y7" s="18"/>
+      <c r="Z7" s="19"/>
     </row>
-    <row r="8" spans="1:25" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+    <row r="8" spans="1:26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="9">
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="9">
         <v>0.76</v>
       </c>
-      <c r="G8" s="9"/>
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
       <c r="J8" s="9"/>
-      <c r="K8" s="6"/>
+      <c r="K8" s="9"/>
       <c r="L8" s="6"/>
       <c r="M8" s="6"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="7"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="10"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
       <c r="R8" s="7"/>
-      <c r="S8" s="1"/>
+      <c r="S8" s="7"/>
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
       <c r="W8" s="1"/>
       <c r="X8" s="1"/>
-      <c r="Y8" s="2"/>
+      <c r="Y8" s="1"/>
+      <c r="Z8" s="2"/>
     </row>
-    <row r="9" spans="1:25" customFormat="1" ht="30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" customFormat="1" ht="30" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="H9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="I9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="J9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="K9" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="L9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="L9" s="11" t="s">
+      <c r="M9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="M9" s="5" t="s">
+      <c r="N9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="N9" s="5" t="s">
+      <c r="O9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="O9" s="5" t="s">
+      <c r="P9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="P9" s="5" t="s">
+      <c r="Q9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="Q9" s="5" t="s">
+      <c r="R9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="R9" s="5" t="s">
+      <c r="S9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="S9" s="5" t="s">
+      <c r="T9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="T9" s="5" t="s">
+      <c r="U9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="U9" s="4" t="s">
+      <c r="V9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="V9" s="4" t="s">
+      <c r="W9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="W9" s="4" t="s">
+      <c r="X9" s="4" t="s">
         <v>28</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A1:Y1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A6:E7"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="V6:V7"/>
+    <mergeCell ref="A8:F8"/>
     <mergeCell ref="W6:W7"/>
     <mergeCell ref="X6:X7"/>
     <mergeCell ref="Y6:Y7"/>
-    <mergeCell ref="S6:S7"/>
+    <mergeCell ref="Z6:Z7"/>
     <mergeCell ref="T6:T7"/>
     <mergeCell ref="U6:U7"/>
+    <mergeCell ref="V6:V7"/>
+    <mergeCell ref="A1:Z1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A6:F7"/>
+    <mergeCell ref="A5:F5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feature/fsel-5567: Update File Excel
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoKetQuaHocTapAca.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoKetQuaHocTapAca.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PhanPhuc\Fsel\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ManagerReports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ManagerReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC015000-7834-4D5B-9BB2-DA423E8F885D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF9CD7F-C8B9-42FF-8BB8-63C17ACC8AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C9B9EFB7-A784-4396-91D6-1A13258A8575}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="179021" concurrentCalc="0"/>
+  <calcPr calcId="179021"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="59">
   <si>
     <t>BÁO CÁO KẾT QUẢ HỌC TẬP (Academic)</t>
   </si>
@@ -114,21 +114,6 @@
     <t>Ngày hết hạn</t>
   </si>
   <si>
-    <t>30 hs</t>
-  </si>
-  <si>
-    <t>27 hs</t>
-  </si>
-  <si>
-    <t>23 hs</t>
-  </si>
-  <si>
-    <t>18 hs</t>
-  </si>
-  <si>
-    <t>9 hs</t>
-  </si>
-  <si>
     <t>0 hs</t>
   </si>
   <si>
@@ -214,6 +199,9 @@
   </si>
   <si>
     <t>UserName</t>
+  </si>
+  <si>
+    <t>Số điện thoại</t>
   </si>
 </sst>
 </file>
@@ -405,6 +393,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -415,15 +410,8 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -767,67 +755,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-      <c r="P1" s="14"/>
-      <c r="Q1" s="14"/>
-      <c r="R1" s="14"/>
-      <c r="S1" s="14"/>
-      <c r="T1" s="14"/>
-      <c r="U1" s="14"/>
-      <c r="V1" s="14"/>
-      <c r="W1" s="14"/>
-      <c r="X1" s="14"/>
-      <c r="Y1" s="14"/>
-      <c r="Z1" s="14"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
+      <c r="S1" s="17"/>
+      <c r="T1" s="17"/>
+      <c r="U1" s="17"/>
+      <c r="V1" s="17"/>
+      <c r="W1" s="17"/>
+      <c r="X1" s="17"/>
+      <c r="Y1" s="17"/>
+      <c r="Z1" s="17"/>
     </row>
     <row r="2" spans="1:26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
       <c r="G2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="H2" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="N2" s="6" t="s">
         <v>38</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>43</v>
       </c>
       <c r="O2" s="6"/>
       <c r="P2" s="6"/>
@@ -843,16 +831,16 @@
       <c r="Z2" s="2"/>
     </row>
     <row r="3" spans="1:26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
       <c r="G3" s="6">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="H3" s="6"/>
       <c r="I3" s="6"/>
@@ -875,31 +863,31 @@
       <c r="Z3" s="2"/>
     </row>
     <row r="4" spans="1:26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
       <c r="G4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="L4" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="K4" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>49</v>
       </c>
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
@@ -917,16 +905,16 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="5" spans="1:26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
+      <c r="A5" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
       <c r="G5" s="6" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="H5" s="6"/>
       <c r="I5" s="6"/>
@@ -949,122 +937,122 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6" spans="1:26" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
       <c r="G6" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="N6" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="O6" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="P6" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="Q6" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="J6" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="K6" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="L6" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="M6" s="8" t="s">
+      <c r="R6" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="N6" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="O6" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="P6" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q6" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="R6" s="8" t="s">
-        <v>61</v>
-      </c>
       <c r="S6" s="8"/>
-      <c r="T6" s="18"/>
-      <c r="U6" s="18"/>
-      <c r="V6" s="18"/>
-      <c r="W6" s="18"/>
-      <c r="X6" s="18"/>
-      <c r="Y6" s="18"/>
-      <c r="Z6" s="19"/>
+      <c r="T6" s="14"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="14"/>
+      <c r="W6" s="14"/>
+      <c r="X6" s="14"/>
+      <c r="Y6" s="14"/>
+      <c r="Z6" s="15"/>
     </row>
     <row r="7" spans="1:26" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="17"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
+      <c r="A7" s="19"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
       <c r="G7" s="8" t="s">
         <v>29</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="L7" s="8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="M7" s="8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="N7" s="8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="P7" s="8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="Q7" s="8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="R7" s="8" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="S7" s="8"/>
-      <c r="T7" s="18"/>
-      <c r="U7" s="18"/>
-      <c r="V7" s="18"/>
-      <c r="W7" s="18"/>
-      <c r="X7" s="18"/>
-      <c r="Y7" s="18"/>
-      <c r="Z7" s="19"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14"/>
+      <c r="V7" s="14"/>
+      <c r="W7" s="14"/>
+      <c r="X7" s="14"/>
+      <c r="Y7" s="14"/>
+      <c r="Z7" s="15"/>
     </row>
     <row r="8" spans="1:26" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
       <c r="G8" s="9">
-        <v>0.76</v>
+        <v>0</v>
       </c>
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
@@ -1091,13 +1079,13 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>1</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>9</v>
@@ -1162,6 +1150,12 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A1:Z1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A6:F7"/>
+    <mergeCell ref="A5:F5"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="W6:W7"/>
     <mergeCell ref="X6:X7"/>
@@ -1170,12 +1164,6 @@
     <mergeCell ref="T6:T7"/>
     <mergeCell ref="U6:U7"/>
     <mergeCell ref="V6:V7"/>
-    <mergeCell ref="A1:Z1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A6:F7"/>
-    <mergeCell ref="A5:F5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>